<commit_message>
git commit "Product stock Admin V2"
</commit_message>
<xml_diff>
--- a/ZlaataQA/reports/Extent-Report/Zlaata-QAResults.xlsx
+++ b/ZlaataQA/reports/Extent-Report/Zlaata-QAResults.xlsx
@@ -189,37 +189,37 @@
     <t>device</t>
   </si>
   <si>
-    <t>Jul 02, 2026 3:54:15 PM</t>
+    <t>Jul 20, 2026 12:04:35 pm</t>
   </si>
   <si>
-    <t>Jul 02, 2026 3:53:33 PM</t>
+    <t>Jul 20, 2026 12:01:04 pm</t>
   </si>
   <si>
-    <t>Jul 02, 2026 3:54:13 PM</t>
+    <t>Jul 20, 2026 12:04:34 pm</t>
   </si>
   <si>
-    <t>40.048 s</t>
+    <t>3 m 30.421 s</t>
   </si>
   <si>
     <t>100%</t>
   </si>
   <si>
-    <t>TC_UI_Zlaata_Raw_01 |Verify admin can add a new raw material successfully.|"TD_UI_Zlaata_Raw_01"</t>
+    <t>TC_UI_Zlaata_PS_03 |Verify that the low stock alert is saved and reflected successfully for the product.| "TD_UI_Zlaata_PS_03"</t>
   </si>
   <si>
-    <t>39.192 s</t>
+    <t>3 m 29.699 s</t>
   </si>
   <si>
-    <t>Raw Material Management</t>
+    <t>Product Stock Management</t>
   </si>
   <si>
-    <t>@TC_UI_Zlaata_Raw_01</t>
+    <t>@TC_UI_Zlaata_PS_03</t>
   </si>
   <si>
-    <t>@Regression</t>
+    <t>@PS</t>
   </si>
   <si>
-    <t>39.199 s</t>
+    <t>3 m 29.703 s</t>
   </si>
 </sst>
 </file>
@@ -1791,7 +1791,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>TC_UI_Zlaata_Raw_01 |Verify admin can add a new raw material successfully.|"TD_UI_Zlaata_Raw_01"</c:v>
+                  <c:v>TC_UI_Zlaata_PS_03 |Verify that the low stock alert is saved and reflected successfully for the product.| "TD_UI_Zlaata_PS_03"</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1802,7 +1802,7 @@
               <c:numCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>2.0</c:v>
+                  <c:v>3.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1863,7 +1863,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>TC_UI_Zlaata_Raw_01 |Verify admin can add a new raw material successfully.|"TD_UI_Zlaata_Raw_01"</c:v>
+                  <c:v>TC_UI_Zlaata_PS_03 |Verify that the low stock alert is saved and reflected successfully for the product.| "TD_UI_Zlaata_PS_03"</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1930,7 +1930,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>TC_UI_Zlaata_Raw_01 |Verify admin can add a new raw material successfully.|"TD_UI_Zlaata_Raw_01"</c:v>
+                  <c:v>TC_UI_Zlaata_PS_03 |Verify that the low stock alert is saved and reflected successfully for the product.| "TD_UI_Zlaata_PS_03"</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2337,10 +2337,10 @@
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>@TC_UI_Zlaata_Raw_01</c:v>
+                  <c:v>@TC_UI_Zlaata_PS_03</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>@Regression</c:v>
+                  <c:v>@PS</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2416,10 +2416,10 @@
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>@TC_UI_Zlaata_Raw_01</c:v>
+                  <c:v>@TC_UI_Zlaata_PS_03</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>@Regression</c:v>
+                  <c:v>@PS</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2487,10 +2487,10 @@
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>@TC_UI_Zlaata_Raw_01</c:v>
+                  <c:v>@TC_UI_Zlaata_PS_03</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>@Regression</c:v>
+                  <c:v>@PS</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2706,7 +2706,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Raw Material Management</c:v>
+                  <c:v>Product Stock Management</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2778,7 +2778,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Raw Material Management</c:v>
+                  <c:v>Product Stock Management</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2845,7 +2845,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Raw Material Management</c:v>
+                  <c:v>Product Stock Management</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5785,7 +5785,7 @@
     <col min="7" max="7" customWidth="true" width="20.85546875"/>
   </cols>
   <sheetData/>
-  <sheetProtection sheet="true" password="E099" scenarios="true" objects="true"/>
+  <sheetProtection sheet="true" password="854B" scenarios="true" objects="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -5869,10 +5869,10 @@
         <v>29</v>
       </c>
       <c r="G22" s="57" t="n">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="H22" s="58" t="n">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="I22" s="59"/>
       <c r="J22" s="60"/>
@@ -6128,10 +6128,10 @@
         <v>54</v>
       </c>
       <c r="J22" s="57" t="n">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="K22" s="58" t="n">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="L22" s="59"/>
       <c r="M22" s="60"/>
@@ -6205,7 +6205,7 @@
         <v>12</v>
       </c>
       <c r="H2" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -6274,7 +6274,7 @@
       </c>
       <c r="H5" t="n" s="0">
         <f>SUM(H2:H4)</f>
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>